<commit_message>
docs/workbook: clarify the calibration-basis delta; remove overlapping merges in Mass_Summary
- READMEs: the declared delta also admits the 17 rigorously checked <inertial> blocks.
- Canonical workbook: removed the redundant overlapping merged ranges of Mass_Summary (present in the
  original file, flagged by a final OpenXML structural check); no value or formula changes.
  Manifest entry, immutability pin and report hashes updated accordingly.
- No change to calibration logic, URDF, meshes or firmware.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
+++ b/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
@@ -8335,10 +8335,6 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A13:F13"/>
-    <x:mergeCell ref="A13:F14"/>
-    <x:mergeCell ref="A1:B1"/>
-    <x:mergeCell ref="A2:B2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
workbook: align JointParametersTable column names with the approved header cells
The approved workbook (68e64ce0…a546) renamed three header cells of
Joint_Parameters row 7 (U, W, X: "Tetto a vuoto 3S [ RPM ]" and "Budget coppia
3S" [kg·cm]/[N·m]) but left the table definition (xl/tables/table1.xml) with the
old names (Speed [rpm], Torque [kg·cm], Effort [N·m]). Excel requires the
header cells to match the table columns and would offer to repair the file.

Only xl/tables/table1.xml changes (the three tableColumn names). Sheets,
formulas, values, styles and the chart are byte-identical to the approved file.
New workbook SHA-256 f376b42f…1827; manifest and its test pin updated. The
approved bytes stay in the previous commit; `git revert` of this commit
restores them.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
+++ b/03_CAD/URDF/matt_robodog_rev00/reference/Coordinate_Cinematiche_matt_robodog_rev00.xlsx
@@ -1722,10 +1722,10 @@
     <x:tableColumn id="18" name="Z parent&#10;[m]"/>
     <x:tableColumn id="19" name="θ min&#10;[rad]"/>
     <x:tableColumn id="20" name="θ max&#10;[rad]"/>
-    <x:tableColumn id="21" name="Speed&#10;[rpm]"/>
+    <x:tableColumn id="21" name="Tetto a vuoto 3S&#10;[ RPM ]"/>
     <x:tableColumn id="22" name="Speed&#10;[rad/s]"/>
-    <x:tableColumn id="23" name="Torque&#10;[kg·cm]"/>
-    <x:tableColumn id="24" name="Effort&#10;[N·m]"/>
+    <x:tableColumn id="23" name="Budget coppia 3S&#10;[kg·cm]"/>
+    <x:tableColumn id="24" name="Budget coppia 3S&#10;[N·m]"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </x:table>

</xml_diff>